<commit_message>
(render and softdelete) :- added softdelete feature and update render-reload logic accordingly
</commit_message>
<xml_diff>
--- a/Database/MyApp-MVC Store Procedure.xlsx
+++ b/Database/MyApp-MVC Store Procedure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\WebApi projects\MyApp-MVC\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32D2EE67-95BA-4F36-87F0-2A458E8287DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5BE68B-0576-4752-BFD9-D6DC384243C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AB8B7940-4CC8-4898-B53F-5686EB1974E8}"/>
   </bookViews>
@@ -41,30 +41,10 @@
     <t>sp_CreateItem</t>
   </si>
   <si>
-    <t>USE MyApp;
-GO
-create procedure sp_CreateItem
-	@Name nvarchar(100),
-	@Price float
-as
-Begin
-	insert into Items values(@Name,@Price);
-end;</t>
-  </si>
-  <si>
     <t>SP Names</t>
   </si>
   <si>
     <t>SP SQL</t>
-  </si>
-  <si>
-    <t>USE MyApp;
-GO
-create procedure sp_GetAllItems
-as
-Begin
-	select Id,Name,Price from Items;
-end;</t>
   </si>
   <si>
     <t>sp_GetAllItems</t>
@@ -98,17 +78,37 @@
     <t>sp_UpdateItem</t>
   </si>
   <si>
-    <t>USE MyApp;
-GO
-create procedure sp_DeleteItem
-	@id int
+    <t>sp_DeleteItem</t>
+  </si>
+  <si>
+    <t>Use MyApp
+Go 
+Alter procedure sp_DeleteItem
+	@Id int
 as
 Begin
-	delete from Items where Id=@id;
+	update items set IsDeleted=1 where Id=@id;
 end;</t>
   </si>
   <si>
-    <t>sp_DeleteItem</t>
+    <t>ALTER PROCEDURE sp_CreateItem
+    @Name NVARCHAR(100),
+    @Price FLOAT
+AS
+BEGIN
+    SET NOCOUNT ON;
+    INSERT INTO Items (Name, Price)
+    VALUES (@Name, @Price);
+END;</t>
+  </si>
+  <si>
+    <t>ALTER PROCEDURE sp_GetAllItems
+AS
+BEGIN
+    SELECT Id, Name, Price
+    FROM Items
+    WHERE IsDeleted = 0;
+END;</t>
   </si>
 </sst>
 </file>
@@ -506,50 +506,50 @@
   <sheetData>
     <row r="3" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" ht="129.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="2:3" ht="144" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="2:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="144" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="115.2" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
(merge create & update):-merge update and create endpoint to save items and create seprate dto,repo,service method and remove create and update methods
</commit_message>
<xml_diff>
--- a/Database/MyApp-MVC Store Procedure.xlsx
+++ b/Database/MyApp-MVC Store Procedure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\WebApi projects\MyApp-MVC\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5BE68B-0576-4752-BFD9-D6DC384243C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DAA064-EA90-436A-A9D7-CCA0180A1686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AB8B7940-4CC8-4898-B53F-5686EB1974E8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>sp_CreateItem</t>
   </si>
@@ -108,6 +108,33 @@
     SELECT Id, Name, Price
     FROM Items
     WHERE IsDeleted = 0;
+END;</t>
+  </si>
+  <si>
+    <t>sp_SaveItem</t>
+  </si>
+  <si>
+    <t>ALTER PROCEDURE sp_SaveItem
+    @Id INT = NULL,
+    @Name NVARCHAR(100),
+    @Price FLOAT
+AS
+BEGIN
+    SET NOCOUNT ON;
+    IF @Id IS NULL OR @Id = 0
+    BEGIN
+        INSERT INTO Items (Name, Price)
+        VALUES (@Name, @Price);
+        SELECT CAST(SCOPE_IDENTITY() AS INT) AS Id; 
+    END
+    ELSE
+    BEGIN
+        UPDATE Items
+        SET Name = @Name,
+            Price = @Price
+        WHERE Id = @Id AND IsDeleted = 0;
+        SELECT @Id AS Id; 
+    END
 END;</t>
   </si>
 </sst>
@@ -152,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -162,6 +189,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -552,8 +582,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B9" s="2"/>
+    <row r="9" spans="2:3" ht="360" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="10" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>

</xml_diff>